<commit_message>
Added eval 15 to delegation table
</commit_message>
<xml_diff>
--- a/dashboard-ui/src/components/SurveyResults/Survey Delegation Variables.xlsx
+++ b/dashboard-ui/src/components/SurveyResults/Survey Delegation Variables.xlsx
@@ -1,15 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29127"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gary.cheng_cn\Projects\itm-evaluation-dashboard\dashboard-ui\src\components\SurveyResults\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7A6B4C5-2DF6-4E99-9037-EC30EEC7ED99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
+    <workbookView xWindow="-140" yWindow="0" windowWidth="19260" windowHeight="12090" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet r:id="rId1" sheetId="1" name="Sheet1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
@@ -151,9 +157,6 @@
     <t>The total time it took the participant to read through the instructions</t>
   </si>
   <si>
-    <t>X refers to the block number, Y refers to the DM number the participant saw. For Eval 4 and 5, participants saw 4 blocks with 2-3 DMs each. The following columns describe each page of the survey using this BX_DMY format.</t>
-  </si>
-  <si>
     <t>The TA1 team that made the scenario the DM responded to</t>
   </si>
   <si>
@@ -224,9 +227,6 @@
   </si>
   <si>
     <r>
-      <t/>
-    </r>
-    <r>
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
@@ -239,7 +239,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -259,7 +259,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -279,7 +279,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -299,7 +299,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -331,9 +331,6 @@
   </si>
   <si>
     <r>
-      <t/>
-    </r>
-    <r>
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
@@ -346,7 +343,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -369,9 +366,6 @@
   </si>
   <si>
     <r>
-      <t/>
-    </r>
-    <r>
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
@@ -384,7 +378,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -404,7 +398,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -424,7 +418,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -444,7 +438,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -464,9 +458,6 @@
   </si>
   <si>
     <r>
-      <t/>
-    </r>
-    <r>
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
@@ -479,7 +470,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -499,7 +490,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -519,7 +510,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -539,7 +530,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -559,9 +550,6 @@
   </si>
   <si>
     <r>
-      <t/>
-    </r>
-    <r>
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
@@ -574,7 +562,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -594,7 +582,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -614,7 +602,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -634,7 +622,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -654,9 +642,6 @@
   </si>
   <si>
     <r>
-      <t/>
-    </r>
-    <r>
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
@@ -669,7 +654,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -689,7 +674,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -709,7 +694,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -729,7 +714,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -749,9 +734,6 @@
   </si>
   <si>
     <r>
-      <t/>
-    </r>
-    <r>
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
@@ -764,7 +746,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -784,7 +766,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -804,7 +786,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -824,7 +806,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -844,9 +826,6 @@
   </si>
   <si>
     <r>
-      <t/>
-    </r>
-    <r>
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
@@ -859,7 +838,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -879,7 +858,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -899,7 +878,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -919,7 +898,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -936,14 +915,16 @@
       </rPr>
       <t xml:space="preserve"> 5 - Completely confident</t>
     </r>
+  </si>
+  <si>
+    <t>X refers to the block number, Y refers to the DM number the participant saw. For Eval 15, participants saw 5 blocks with 2-3 DMs each (multi-KDMA blocks have aligned and baseline; the single MF block also includes misaligned). The following columns describe each page of the survey using this BX_DMY format.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
-  <numFmts count="0"/>
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -956,6 +937,20 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -986,34 +981,35 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="7">
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" builtinId="0" name="Normal"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14ac:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1024,10 +1020,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr lastClr="000000" val="windowText"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr lastClr="FFFFFF" val="window"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="44546A"/>
@@ -1065,71 +1061,71 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Times New Roman" script="Arab"/>
-        <a:font typeface="Times New Roman" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="MoolBoran" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Times New Roman" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Arial" script="Arab"/>
-        <a:font typeface="Arial" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="DaunPenh" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Arial" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -1157,7 +1153,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -1180,11 +1176,11 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="9525">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="9500"/>
@@ -1193,13 +1189,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="25400">
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="38100">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -1209,7 +1205,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -1218,7 +1214,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -1227,7 +1223,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -1235,10 +1231,10 @@
           </a:effectLst>
           <a:scene3d>
             <a:camera prst="orthographicFront">
-              <a:rot rev="0" lon="0" lat="0"/>
+              <a:rot lat="0" lon="0" rev="0"/>
             </a:camera>
-            <a:lightRig dir="t" rig="threePt">
-              <a:rot rev="1200000" lon="0" lat="0"/>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
             </a:lightRig>
           </a:scene3d>
           <a:sp3d>
@@ -1303,51 +1299,39 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:AI3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="6" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="6" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="6" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="16" max="16" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="17" max="17" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="18" max="18" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="19" max="19" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="20" max="20" style="6" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="21" max="21" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="22" max="22" style="5" width="19.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="23" max="23" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="24" max="24" style="5" width="20.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="25" max="25" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="26" max="26" style="5" width="18.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="27" max="27" style="5" width="18.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="28" max="28" style="5" width="18.14785714285714" customWidth="1" bestFit="1"/>
-    <col min="29" max="29" style="5" width="19.433571428571426" customWidth="1" bestFit="1"/>
-    <col min="30" max="30" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="31" max="31" style="5" width="22.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="32" max="32" style="5" width="25.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="33" max="33" style="5" width="18.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="34" max="34" style="5" width="23.005" customWidth="1" bestFit="1"/>
-    <col min="35" max="35" style="5" width="25.005" customWidth="1" bestFit="1"/>
+    <col min="1" max="6" width="16.7265625" style="5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.453125" style="6" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.7265625" style="5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.453125" style="6" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="16.7265625" style="5" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.453125" style="6" bestFit="1" customWidth="1"/>
+    <col min="13" max="19" width="16.7265625" style="5" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="12.453125" style="6" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="16.7265625" style="5" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="19.81640625" style="5" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="16.7265625" style="5" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="20.26953125" style="5" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="16.7265625" style="5" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="18.7265625" style="5" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="18.54296875" style="5" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="18.1796875" style="5" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="19.453125" style="5" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="16.7265625" style="5" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="22.26953125" style="5" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="25.7265625" style="5" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="18.26953125" style="5" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="23" style="5" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="25" style="5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="46.5" customFormat="1" s="1">
+    <row r="1" spans="1:35" s="1" customFormat="1" ht="46.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1454,7 +1438,7 @@
         <v>34</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="208.5" customFormat="1" s="1">
+    <row r="2" spans="1:35" s="1" customFormat="1" ht="208.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>35</v>
       </c>
@@ -1492,82 +1476,82 @@
         <v>44</v>
       </c>
       <c r="M2" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="N2" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="N2" s="2" t="s">
+      <c r="O2" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="O2" s="2" t="s">
+      <c r="P2" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="P2" s="2" t="s">
+      <c r="Q2" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="Q2" s="2" t="s">
+      <c r="R2" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="R2" s="2" t="s">
+      <c r="S2" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="S2" s="2" t="s">
+      <c r="T2" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="T2" s="3" t="s">
+      <c r="U2" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="U2" s="2" t="s">
+      <c r="V2" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="V2" s="2" t="s">
+      <c r="W2" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="W2" s="2" t="s">
+      <c r="X2" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="X2" s="2" t="s">
+      <c r="Y2" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="Y2" s="2" t="s">
+      <c r="Z2" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="Z2" s="2" t="s">
+      <c r="AA2" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="AA2" s="2" t="s">
+      <c r="AB2" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="AB2" s="2" t="s">
+      <c r="AC2" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="AC2" s="2" t="s">
+      <c r="AD2" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="AD2" s="2" t="s">
+      <c r="AE2" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="AE2" s="2" t="s">
+      <c r="AF2" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="AF2" s="2" t="s">
+      <c r="AG2" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="AG2" s="2" t="s">
+      <c r="AH2" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="AH2" s="2" t="s">
+      <c r="AI2" s="2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="3" spans="1:35" s="1" customFormat="1" ht="114" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="2" t="s">
         <v>66</v>
-      </c>
-      <c r="AI2" s="2" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="114" customFormat="1" s="1">
-      <c r="A3" s="2" t="s">
-        <v>67</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D3" s="2"/>
       <c r="E3" s="4"/>
@@ -1576,42 +1560,42 @@
       <c r="H3" s="2"/>
       <c r="I3" s="3"/>
       <c r="J3" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K3" s="2"/>
       <c r="L3" s="3"/>
       <c r="M3" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="N3" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="N3" s="2" t="s">
+      <c r="O3" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="O3" s="2" t="s">
+      <c r="P3" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="P3" s="2" t="s">
+      <c r="Q3" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="Q3" s="2" t="s">
+      <c r="R3" s="2" t="s">
         <v>74</v>
-      </c>
-      <c r="R3" s="2" t="s">
-        <v>75</v>
       </c>
       <c r="S3" s="2"/>
       <c r="T3" s="3"/>
       <c r="U3" s="2"/>
       <c r="V3" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="W3" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="W3" s="2" t="s">
+      <c r="X3" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="X3" s="2" t="s">
+      <c r="Y3" s="2" t="s">
         <v>78</v>
-      </c>
-      <c r="Y3" s="2" t="s">
-        <v>79</v>
       </c>
       <c r="Z3" s="2"/>
       <c r="AA3" s="2"/>
@@ -1619,12 +1603,12 @@
       <c r="AC3" s="2"/>
       <c r="AD3" s="2"/>
       <c r="AE3" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="AF3" s="2"/>
       <c r="AG3" s="2"/>
       <c r="AH3" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="AI3" s="2"/>
     </row>

</xml_diff>

<commit_message>
Revert survey delegation variables file
</commit_message>
<xml_diff>
--- a/dashboard-ui/src/components/SurveyResults/Survey Delegation Variables.xlsx
+++ b/dashboard-ui/src/components/SurveyResults/Survey Delegation Variables.xlsx
@@ -1,21 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29127"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gary.cheng_cn\Projects\itm-evaluation-dashboard\dashboard-ui\src\components\SurveyResults\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7A6B4C5-2DF6-4E99-9037-EC30EEC7ED99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-140" yWindow="0" windowWidth="19260" windowHeight="12090" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet r:id="rId1" sheetId="1" name="Sheet1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -157,6 +151,9 @@
     <t>The total time it took the participant to read through the instructions</t>
   </si>
   <si>
+    <t>X refers to the block number, Y refers to the DM number the participant saw. For Eval 4 and 5, participants saw 4 blocks with 2-3 DMs each. The following columns describe each page of the survey using this BX_DMY format.</t>
+  </si>
+  <si>
     <t>The TA1 team that made the scenario the DM responded to</t>
   </si>
   <si>
@@ -227,6 +224,9 @@
   </si>
   <si>
     <r>
+      <t/>
+    </r>
+    <r>
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
@@ -239,7 +239,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -259,7 +259,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -279,7 +279,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -299,7 +299,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -331,6 +331,9 @@
   </si>
   <si>
     <r>
+      <t/>
+    </r>
+    <r>
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
@@ -343,7 +346,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -366,6 +369,9 @@
   </si>
   <si>
     <r>
+      <t/>
+    </r>
+    <r>
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
@@ -378,7 +384,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -398,7 +404,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -418,7 +424,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -438,7 +444,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -458,6 +464,9 @@
   </si>
   <si>
     <r>
+      <t/>
+    </r>
+    <r>
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
@@ -470,7 +479,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -490,7 +499,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -510,7 +519,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -530,7 +539,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -550,6 +559,9 @@
   </si>
   <si>
     <r>
+      <t/>
+    </r>
+    <r>
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
@@ -562,7 +574,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -582,7 +594,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -602,7 +614,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -622,7 +634,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -642,6 +654,9 @@
   </si>
   <si>
     <r>
+      <t/>
+    </r>
+    <r>
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
@@ -654,7 +669,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -674,7 +689,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -694,7 +709,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -714,7 +729,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -734,6 +749,9 @@
   </si>
   <si>
     <r>
+      <t/>
+    </r>
+    <r>
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
@@ -746,7 +764,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -766,7 +784,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -786,7 +804,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -806,7 +824,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -826,6 +844,9 @@
   </si>
   <si>
     <r>
+      <t/>
+    </r>
+    <r>
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
@@ -838,7 +859,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -858,7 +879,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -878,7 +899,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -898,7 +919,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -915,16 +936,14 @@
       </rPr>
       <t xml:space="preserve"> 5 - Completely confident</t>
     </r>
-  </si>
-  <si>
-    <t>X refers to the block number, Y refers to the DM number the participant saw. For Eval 15, participants saw 5 blocks with 2-3 DMs each (multi-KDMA blocks have aligned and baseline; the single MF block also includes misaligned). The following columns describe each page of the survey using this BX_DMY format.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
+  <numFmts count="0"/>
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -937,20 +956,6 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -981,35 +986,34 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="7">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle xfId="0" builtinId="0" name="Normal"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14ac:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1020,10 +1024,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
+        <a:sysClr lastClr="000000" val="windowText"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
+        <a:sysClr lastClr="FFFFFF" val="window"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="44546A"/>
@@ -1061,71 +1065,71 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
+        <a:font typeface="맑은 고딕" script="Hang"/>
+        <a:font typeface="宋体" script="Hans"/>
+        <a:font typeface="新細明體" script="Hant"/>
+        <a:font typeface="Times New Roman" script="Arab"/>
+        <a:font typeface="Times New Roman" script="Hebr"/>
+        <a:font typeface="Tahoma" script="Thai"/>
+        <a:font typeface="Nyala" script="Ethi"/>
+        <a:font typeface="Vrinda" script="Beng"/>
+        <a:font typeface="Shruti" script="Gujr"/>
+        <a:font typeface="MoolBoran" script="Khmr"/>
+        <a:font typeface="Tunga" script="Knda"/>
+        <a:font typeface="Raavi" script="Guru"/>
+        <a:font typeface="Euphemia" script="Cans"/>
+        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
+        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
+        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
+        <a:font typeface="MV Boli" script="Thaa"/>
+        <a:font typeface="Mangal" script="Deva"/>
+        <a:font typeface="Gautami" script="Telu"/>
+        <a:font typeface="Latha" script="Taml"/>
+        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
+        <a:font typeface="Kalinga" script="Orya"/>
+        <a:font typeface="Kartika" script="Mlym"/>
+        <a:font typeface="DokChampa" script="Laoo"/>
+        <a:font typeface="Iskoola Pota" script="Sinh"/>
+        <a:font typeface="Mongolian Baiti" script="Mong"/>
+        <a:font typeface="Times New Roman" script="Viet"/>
+        <a:font typeface="Microsoft Uighur" script="Uigh"/>
+        <a:font typeface="Sylfaen" script="Geor"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
+        <a:font typeface="맑은 고딕" script="Hang"/>
+        <a:font typeface="宋体" script="Hans"/>
+        <a:font typeface="新細明體" script="Hant"/>
+        <a:font typeface="Arial" script="Arab"/>
+        <a:font typeface="Arial" script="Hebr"/>
+        <a:font typeface="Tahoma" script="Thai"/>
+        <a:font typeface="Nyala" script="Ethi"/>
+        <a:font typeface="Vrinda" script="Beng"/>
+        <a:font typeface="Shruti" script="Gujr"/>
+        <a:font typeface="DaunPenh" script="Khmr"/>
+        <a:font typeface="Tunga" script="Knda"/>
+        <a:font typeface="Raavi" script="Guru"/>
+        <a:font typeface="Euphemia" script="Cans"/>
+        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
+        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
+        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
+        <a:font typeface="MV Boli" script="Thaa"/>
+        <a:font typeface="Mangal" script="Deva"/>
+        <a:font typeface="Gautami" script="Telu"/>
+        <a:font typeface="Latha" script="Taml"/>
+        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
+        <a:font typeface="Kalinga" script="Orya"/>
+        <a:font typeface="Kartika" script="Mlym"/>
+        <a:font typeface="DokChampa" script="Laoo"/>
+        <a:font typeface="Iskoola Pota" script="Sinh"/>
+        <a:font typeface="Mongolian Baiti" script="Mong"/>
+        <a:font typeface="Arial" script="Viet"/>
+        <a:font typeface="Microsoft Uighur" script="Uigh"/>
+        <a:font typeface="Sylfaen" script="Geor"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -1153,7 +1157,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
+          <a:lin scaled="1" ang="16200000"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -1176,11 +1180,11 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
+          <a:lin scaled="1" ang="16200000"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="9525">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="9500"/>
@@ -1189,13 +1193,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="25400">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="38100">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -1205,7 +1209,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -1214,7 +1218,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -1223,7 +1227,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -1231,10 +1235,10 @@
           </a:effectLst>
           <a:scene3d>
             <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
+              <a:rot rev="0" lon="0" lat="0"/>
             </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
+            <a:lightRig dir="t" rig="threePt">
+              <a:rot rev="1200000" lon="0" lat="0"/>
             </a:lightRig>
           </a:scene3d>
           <a:sp3d>
@@ -1299,39 +1303,51 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:AI3"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="6" width="16.7265625" style="5" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.453125" style="6" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.7265625" style="5" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.453125" style="6" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="16.7265625" style="5" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.453125" style="6" bestFit="1" customWidth="1"/>
-    <col min="13" max="19" width="16.7265625" style="5" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12.453125" style="6" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="16.7265625" style="5" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="19.81640625" style="5" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="16.7265625" style="5" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="20.26953125" style="5" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="16.7265625" style="5" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="18.7265625" style="5" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="18.54296875" style="5" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="18.1796875" style="5" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="19.453125" style="5" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="16.7265625" style="5" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="22.26953125" style="5" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="25.7265625" style="5" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="18.26953125" style="5" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="23" style="5" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="25" style="5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="6" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="6" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="6" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="17" max="17" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="18" max="18" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="19" max="19" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="20" max="20" style="6" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="21" max="21" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="22" max="22" style="5" width="19.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="23" max="23" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="24" max="24" style="5" width="20.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="25" max="25" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="26" max="26" style="5" width="18.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="27" max="27" style="5" width="18.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="28" max="28" style="5" width="18.14785714285714" customWidth="1" bestFit="1"/>
+    <col min="29" max="29" style="5" width="19.433571428571426" customWidth="1" bestFit="1"/>
+    <col min="30" max="30" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="31" max="31" style="5" width="22.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="32" max="32" style="5" width="25.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="33" max="33" style="5" width="18.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="34" max="34" style="5" width="23.005" customWidth="1" bestFit="1"/>
+    <col min="35" max="35" style="5" width="25.005" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" s="1" customFormat="1" ht="46.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="46.5" customFormat="1" s="1">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1438,7 +1454,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="2" spans="1:35" s="1" customFormat="1" ht="208.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="208.5" customFormat="1" s="1">
       <c r="A2" s="2" t="s">
         <v>35</v>
       </c>
@@ -1476,82 +1492,82 @@
         <v>44</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>81</v>
+        <v>45</v>
       </c>
       <c r="N2" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="O2" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="P2" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="Q2" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="R2" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="S2" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="T2" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="U2" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="V2" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="W2" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="X2" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="Y2" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Z2" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="AA2" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="AB2" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="AC2" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="AD2" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="AE2" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="AF2" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="AG2" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="AH2" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="AI2" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="AH2" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="AI2" s="2" t="s">
-        <v>63</v>
-      </c>
     </row>
-    <row r="3" spans="1:35" s="1" customFormat="1" ht="114" customHeight="1" x14ac:dyDescent="0.35">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="114" customFormat="1" s="1">
       <c r="A3" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D3" s="2"/>
       <c r="E3" s="4"/>
@@ -1560,42 +1576,42 @@
       <c r="H3" s="2"/>
       <c r="I3" s="3"/>
       <c r="J3" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="K3" s="2"/>
       <c r="L3" s="3"/>
       <c r="M3" s="2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="O3" s="2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="P3" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Q3" s="2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="R3" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="S3" s="2"/>
       <c r="T3" s="3"/>
       <c r="U3" s="2"/>
       <c r="V3" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="W3" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="X3" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="Y3" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="Z3" s="2"/>
       <c r="AA3" s="2"/>
@@ -1603,12 +1619,12 @@
       <c r="AC3" s="2"/>
       <c r="AD3" s="2"/>
       <c r="AE3" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="AF3" s="2"/>
       <c r="AG3" s="2"/>
       <c r="AH3" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="AI3" s="2"/>
     </row>

</xml_diff>